<commit_message>
Blank Slate: regenerate deck + workbook with title-scan fixes
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/decks/blank-slate/keyword-research.xlsx
+++ b/decks/blank-slate/keyword-research.xlsx
@@ -795,7 +795,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Closing the Knowledge Gap in New Employee Compliance Training</t>
+          <t>New Employee Compliance Training When the Pressure Is On</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
@@ -846,7 +846,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Evaluating Corporate Compliance Training Solutions for Zero-Fail Teams</t>
+          <t>Evaluating Corporate Compliance Training Solutions for High-Stakes Teams</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
@@ -897,7 +897,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Measuring What Compliance Training for New Employees Really Delivers</t>
+          <t>Compliance Training for New Employees: Where Most Programs Break Down</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -948,7 +948,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Making Training Compliance Tracking Stick for Zero-Fail Teams</t>
+          <t>Training Compliance Tracking: Retention Over Completion</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -1050,7 +1050,7 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Why Interactive Training Won't Stick Without Reinforcement</t>
+          <t>The Science Behind Interactive Training</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
@@ -1097,7 +1097,7 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Turning Motivational Training Into Readiness You Can Prove</t>
+          <t>Why Motivational Training Won't Stick Without Reinforcement</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
@@ -1148,7 +1148,7 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Motivating Staff Training Without the Training Fatigue</t>
+          <t>Rethinking Motivating Staff Training for Safety-Critical Teams</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
@@ -1199,7 +1199,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Evaluating Gamification Training Software for Zero-Fail Teams</t>
+          <t>Evaluating Gamification Training Software for Deskless Workforces</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
@@ -1250,7 +1250,7 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Measuring What Corporate Gamification Really Delivers</t>
+          <t>Corporate Gamification: Where Most Programs Break Down</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
@@ -1301,7 +1301,7 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Gamification Features: Retention Over Completion</t>
+          <t>Measuring the Impact of Gamification Features</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
@@ -1348,7 +1348,7 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Gamification Learning Platform: Built for Readiness, Not Completion</t>
+          <t>What Makes a Gamification Platform Actually Work</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
@@ -1450,7 +1450,7 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Turning Microlearning in Corporate Training Into Readiness You Can Prove</t>
+          <t>Why Microlearning in Corporate Training Won't Stick Without Reinforcement</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
@@ -1501,7 +1501,7 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>Rethinking Creating Microlearning Content for Zero-Fail Teams</t>
+          <t>Turning Creating Microlearning Content Into Readiness You Can Prove</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
@@ -1654,7 +1654,7 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>From Checkbox to Capability in Microlearning Strategies</t>
+          <t>Rethinking Microlearning Strategies for Regulated Industries</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
@@ -1705,7 +1705,7 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>Gamified Microlearning That Holds Up Under Pressure</t>
+          <t>Gamified Microlearning Without the Training Fatigue</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
@@ -1756,7 +1756,7 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>Closing the Knowledge Gap in Microlearning Gamification</t>
+          <t>From Checkbox to Capability in Microlearning Gamification</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
@@ -1807,7 +1807,7 @@
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>Measuring What Microlearning Content Development Really Delivers</t>
+          <t>Microlearning Content Development When the Pressure Is On</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
@@ -1905,7 +1905,7 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>Turning Employee Retention Training Into Readiness You Can Prove</t>
+          <t>Employee Retention Training: What Actually Makes It Stick</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
@@ -1956,7 +1956,7 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>Training and Retention: A Readiness-First Approach</t>
+          <t>The Science Behind Training and Retention</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
@@ -2105,7 +2105,7 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>Rethinking Adult Learning Retention for Zero-Fail Teams</t>
+          <t>Why Adult Learning Retention Won't Stick Without Reinforcement</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
@@ -2156,7 +2156,7 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>From Checkbox to Capability in Knowledge Retention After Training</t>
+          <t>Knowledge Retention After Training: A Readiness-First Approach</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
@@ -2207,7 +2207,7 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>Closing the Knowledge Gap in Knowledge Retention in the Workplace</t>
+          <t>Rethinking Knowledge Retention in the Workplace for Zero-Fail Teams</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
@@ -2258,7 +2258,7 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>Measuring What Training Content Development Really Delivers</t>
+          <t>From Checkbox to Capability in Training Content Development</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
@@ -2360,7 +2360,7 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>Why Frontline Leadership Program Won't Stick Without Reinforcement</t>
+          <t>Frontline Leadership Program: Retention Over Completion</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
@@ -2411,7 +2411,7 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>Turning Frontline Leadership Course Into Readiness You Can Prove</t>
+          <t>Making Frontline Leadership Course Stick for High-Stakes Teams</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
@@ -2462,7 +2462,7 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>Training for Frontline Staff That Holds Up Under Pressure</t>
+          <t>Turning Training for Frontline Staff Into Readiness You Can Prove</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
@@ -2513,7 +2513,7 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>External Training Management System: Built to Prove Retention, Not Attendance</t>
+          <t>Choosing External Training Management System for Regulated Industries</t>
         </is>
       </c>
       <c r="C39" s="4" t="inlineStr">
@@ -2564,7 +2564,7 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>Frontline Worker Training: Retention Over Completion</t>
+          <t>Rethinking Frontline Worker Training for Compliance Teams</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr">
@@ -2615,7 +2615,7 @@
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>Making Frontline Leadership Basic Principles Stick for Zero-Fail Teams</t>
+          <t>Frontline Leadership Basic Principles Without the Training Fatigue</t>
         </is>
       </c>
       <c r="C41" s="4" t="inlineStr">
@@ -2764,7 +2764,7 @@
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>Ethics and Compliance Courses That Holds Up Under Pressure</t>
+          <t>Do Your Ethics and Compliance Courses Actually Stick?</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
@@ -2956,7 +2956,7 @@
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>Regulatory Compliance Training Courses: Where Most Programs Break Down</t>
+          <t>Closing the Knowledge Gap in Regulatory Compliance Training Courses</t>
         </is>
       </c>
       <c r="C48" s="4" t="inlineStr">
@@ -3003,7 +3003,7 @@
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>Regulatory Compliance Training Programs: Retention Over Completion</t>
+          <t>Measuring the Impact of Regulatory Compliance Training Programs</t>
         </is>
       </c>
       <c r="C49" s="4" t="inlineStr">
@@ -3050,7 +3050,7 @@
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>Choosing Learning and Development Tools for Zero-Fail Teams</t>
+          <t>Choosing Learning and Development Tools for Compliance Teams</t>
         </is>
       </c>
       <c r="C50" s="4" t="inlineStr">
@@ -3152,7 +3152,7 @@
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>Rethinking Gamification for Employee Engagement for Zero-Fail Teams</t>
+          <t>Gamification for Employee Engagement: A Readiness-First Approach</t>
         </is>
       </c>
       <c r="C52" s="4" t="inlineStr">
@@ -3250,7 +3250,7 @@
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>From Checkbox to Capability in Employee Gamification</t>
+          <t>Employee Gamification Without the Training Fatigue</t>
         </is>
       </c>
       <c r="C54" s="4" t="inlineStr">
@@ -3297,7 +3297,7 @@
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>Employee Engagement Training That Holds Up Under Pressure</t>
+          <t>From Checkbox to Capability in Employee Engagement Training</t>
         </is>
       </c>
       <c r="C55" s="4" t="inlineStr">
@@ -3344,7 +3344,7 @@
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>Making Employee Engagement Training and Development Stick for Zero-Fail Teams</t>
+          <t>Employee Engagement Training and Development: Retention Over Completion</t>
         </is>
       </c>
       <c r="C56" s="4" t="inlineStr">
@@ -3391,7 +3391,7 @@
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>Gamified Features, Reframed for Zero-Fail Teams</t>
+          <t>Making Gamified Features Stick for Zero-Fail Teams</t>
         </is>
       </c>
       <c r="C57" s="4" t="inlineStr">
@@ -3438,7 +3438,7 @@
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>Microlearning Platform: What to Look For</t>
+          <t>Choosing Microlearning Platform for Mission-Critical Teams</t>
         </is>
       </c>
       <c r="C58" s="4" t="inlineStr">
@@ -3489,7 +3489,7 @@
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>Benefits of Microlearning: What Actually Makes It Stick</t>
+          <t>Benefits of Microlearning, Reframed for High-Stakes Teams</t>
         </is>
       </c>
       <c r="C59" s="4" t="inlineStr">
@@ -3536,7 +3536,7 @@
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>Best Microlearning Platforms: Built for Readiness, Not Completion</t>
+          <t>Best Microlearning Platforms: Built to Prove Retention, Not Attendance</t>
         </is>
       </c>
       <c r="C60" s="4" t="inlineStr">
@@ -3587,7 +3587,7 @@
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>Choosing Microlearning Tools for Zero-Fail Teams</t>
+          <t>Evaluating Microlearning Tools for Frontline Teams</t>
         </is>
       </c>
       <c r="C61" s="4" t="inlineStr">
@@ -3638,7 +3638,7 @@
       </c>
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t>The Science Behind Corporate Microlearning</t>
+          <t>Corporate Microlearning: What Actually Makes It Stick</t>
         </is>
       </c>
       <c r="C62" s="4" t="inlineStr">
@@ -3689,7 +3689,7 @@
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t>Microlearning AI: A Readiness-First Approach</t>
+          <t>AI-Powered Microlearning, Explained for Zero-Fail Teams</t>
         </is>
       </c>
       <c r="C63" s="4" t="inlineStr">
@@ -3736,7 +3736,7 @@
       </c>
       <c r="B64" s="3" t="inlineStr">
         <is>
-          <t>Microlearning Modules Without the Training Fatigue</t>
+          <t>Microlearning Modules: A Readiness-First Approach</t>
         </is>
       </c>
       <c r="C64" s="4" t="inlineStr">
@@ -3783,7 +3783,7 @@
       </c>
       <c r="B65" s="3" t="inlineStr">
         <is>
-          <t>Microlearning Resources: Retention Over Completion</t>
+          <t>Closing the Knowledge Gap in Microlearning Resources</t>
         </is>
       </c>
       <c r="C65" s="4" t="inlineStr">
@@ -3830,7 +3830,7 @@
       </c>
       <c r="B66" s="3" t="inlineStr">
         <is>
-          <t>The Buyer's Guide to Spaced Repetition App</t>
+          <t>Choosing Spaced Repetition App for Compliance Teams</t>
         </is>
       </c>
       <c r="C66" s="4" t="inlineStr">
@@ -3881,7 +3881,7 @@
       </c>
       <c r="B67" s="3" t="inlineStr">
         <is>
-          <t>The Science Behind Learning Retention</t>
+          <t>Making Learning Retention Stick for Safety-Critical Teams</t>
         </is>
       </c>
       <c r="C67" s="4" t="inlineStr">
@@ -3928,7 +3928,7 @@
       </c>
       <c r="B68" s="3" t="inlineStr">
         <is>
-          <t>Why Knowledge Retention Won't Stick Without Reinforcement</t>
+          <t>Knowledge Retention, Reframed for Deskless Workforces</t>
         </is>
       </c>
       <c r="C68" s="4" t="inlineStr">
@@ -3975,7 +3975,7 @@
       </c>
       <c r="B69" s="3" t="inlineStr">
         <is>
-          <t>Evaluating Best Spaced Repetition App for Zero-Fail Teams</t>
+          <t>The Buyer's Guide to Best Spaced Repetition App</t>
         </is>
       </c>
       <c r="C69" s="4" t="inlineStr">
@@ -4073,7 +4073,7 @@
       </c>
       <c r="B71" s="3" t="inlineStr">
         <is>
-          <t>Knowledge Retention Strategies Without the Training Fatigue</t>
+          <t>Turning Knowledge Retention Strategies Into Readiness You Can Prove</t>
         </is>
       </c>
       <c r="C71" s="4" t="inlineStr">
@@ -4214,7 +4214,7 @@
       </c>
       <c r="B74" s="3" t="inlineStr">
         <is>
-          <t>Making Tracking Employee Training Stick for Zero-Fail Teams</t>
+          <t>Closing the Knowledge Gap in Tracking Employee Training</t>
         </is>
       </c>
       <c r="C74" s="4" t="inlineStr">
@@ -4265,7 +4265,7 @@
       </c>
       <c r="B75" s="3" t="inlineStr">
         <is>
-          <t>Frontline Leadership Skills, Reframed for Zero-Fail Teams</t>
+          <t>Frontline Leadership Skills: Where Most Programs Break Down</t>
         </is>
       </c>
       <c r="C75" s="4" t="inlineStr">
@@ -4316,7 +4316,7 @@
       </c>
       <c r="B76" s="3" t="inlineStr">
         <is>
-          <t>Frontline Management Course: A Readiness-First Approach</t>
+          <t>Frontline Management Course, Reframed for Frontline Teams</t>
         </is>
       </c>
       <c r="C76" s="4" t="inlineStr">
@@ -4367,7 +4367,7 @@
       </c>
       <c r="B77" s="3" t="inlineStr">
         <is>
-          <t>Rethinking Frontline Manager Training for Zero-Fail Teams</t>
+          <t>Frontline Manager Training: What Actually Makes It Stick</t>
         </is>
       </c>
       <c r="C77" s="4" t="inlineStr">
@@ -4418,7 +4418,7 @@
       </c>
       <c r="B78" s="3" t="inlineStr">
         <is>
-          <t>Frontline Employee Training: Where Most Programs Break Down</t>
+          <t>Frontline Employee Training: A Readiness-First Approach</t>
         </is>
       </c>
       <c r="C78" s="4" t="inlineStr">
@@ -4865,7 +4865,7 @@
       </c>
       <c r="B87" s="3" t="inlineStr">
         <is>
-          <t>Rethinking HR Compliance Training for Zero-Fail Teams</t>
+          <t>Rethinking HR Compliance Training for Mission-Critical Teams</t>
         </is>
       </c>
       <c r="C87" s="4" t="inlineStr">
@@ -5006,7 +5006,7 @@
       </c>
       <c r="B90" s="3" t="inlineStr">
         <is>
-          <t>Training and Employee Engagement, Reframed for Zero-Fail Teams</t>
+          <t>Making Training and Employee Engagement Stick for Frontline Teams</t>
         </is>
       </c>
       <c r="C90" s="4" t="inlineStr">
@@ -5057,7 +5057,7 @@
       </c>
       <c r="B91" s="3" t="inlineStr">
         <is>
-          <t>Employee Engagement Courses: What Actually Makes It Stick</t>
+          <t>Employee Engagement Courses, Reframed for Regulated Industries</t>
         </is>
       </c>
       <c r="C91" s="4" t="inlineStr">
@@ -5104,7 +5104,7 @@
       </c>
       <c r="B92" s="3" t="inlineStr">
         <is>
-          <t>The Science Behind Gamification in the Workplace</t>
+          <t>Gamification in the Workplace: What Actually Makes It Stick</t>
         </is>
       </c>
       <c r="C92" s="4" t="inlineStr">
@@ -5202,7 +5202,7 @@
       </c>
       <c r="B94" s="3" t="inlineStr">
         <is>
-          <t>Gamified Training: A Readiness-First Approach</t>
+          <t>Turning Gamified Training Into Readiness You Can Prove</t>
         </is>
       </c>
       <c r="C94" s="4" t="inlineStr">
@@ -5300,7 +5300,7 @@
       </c>
       <c r="B96" s="3" t="inlineStr">
         <is>
-          <t>Closing the Knowledge Gap in Interactive Training Modules</t>
+          <t>Interactive Training Modules When the Pressure Is On</t>
         </is>
       </c>
       <c r="C96" s="4" t="inlineStr">
@@ -5347,7 +5347,7 @@
       </c>
       <c r="B97" s="3" t="inlineStr">
         <is>
-          <t>Benefits of Gamification in the Workplace: Where Most Programs Break Down</t>
+          <t>Closing the Knowledge Gap in Benefits of Gamification in the Workplace</t>
         </is>
       </c>
       <c r="C97" s="4" t="inlineStr">
@@ -5394,7 +5394,7 @@
       </c>
       <c r="B98" s="3" t="inlineStr">
         <is>
-          <t>Choosing Microlearning Apps for Zero-Fail Teams</t>
+          <t>Microlearning Apps: Built for Readiness, Not Completion</t>
         </is>
       </c>
       <c r="C98" s="4" t="inlineStr">
@@ -5492,7 +5492,7 @@
       </c>
       <c r="B100" s="3" t="inlineStr">
         <is>
-          <t>The Buyer's Guide to Best Microlearning App</t>
+          <t>Best Microlearning App: What to Look For</t>
         </is>
       </c>
       <c r="C100" s="4" t="inlineStr">
@@ -5543,7 +5543,7 @@
       </c>
       <c r="B101" s="3" t="inlineStr">
         <is>
-          <t>Microlearning Software: Built to Prove Retention, Not Attendance</t>
+          <t>The Buyer's Guide to Microlearning Software</t>
         </is>
       </c>
       <c r="C101" s="4" t="inlineStr">
@@ -5594,7 +5594,7 @@
       </c>
       <c r="B102" s="3" t="inlineStr">
         <is>
-          <t>Evaluating Microlearning Solution for Zero-Fail Teams</t>
+          <t>Choosing a Microlearning Solution for Zero-Fail Teams</t>
         </is>
       </c>
       <c r="C102" s="4" t="inlineStr">
@@ -5692,7 +5692,7 @@
       </c>
       <c r="B104" s="3" t="inlineStr">
         <is>
-          <t>Why LMS Microlearning Won't Stick Without Reinforcement</t>
+          <t>The Science Behind LMS Microlearning</t>
         </is>
       </c>
       <c r="C104" s="4" t="inlineStr">
@@ -5739,7 +5739,7 @@
       </c>
       <c r="B105" s="3" t="inlineStr">
         <is>
-          <t>Microlearning Application: Where Most Programs Break Down</t>
+          <t>Microlearning in Practice: Where It Breaks Down</t>
         </is>
       </c>
       <c r="C105" s="4" t="inlineStr">
@@ -5786,7 +5786,7 @@
       </c>
       <c r="B106" s="3" t="inlineStr">
         <is>
-          <t>Making Spaced Repetition Stick for Zero-Fail Teams</t>
+          <t>Spaced Repetition: Where Most Programs Break Down</t>
         </is>
       </c>
       <c r="C106" s="4" t="inlineStr">
@@ -5837,7 +5837,7 @@
       </c>
       <c r="B107" s="3" t="inlineStr">
         <is>
-          <t>Distributed Practice, Reframed for Zero-Fail Teams</t>
+          <t>Measuring the Impact of Distributed Practice</t>
         </is>
       </c>
       <c r="C107" s="4" t="inlineStr">
@@ -5884,7 +5884,7 @@
       </c>
       <c r="B108" s="3" t="inlineStr">
         <is>
-          <t>Spaced Repetition Software: What to Look For</t>
+          <t>Spaced Repetition Software: Built for Readiness, Not Completion</t>
         </is>
       </c>
       <c r="C108" s="4" t="inlineStr">
@@ -5935,7 +5935,7 @@
       </c>
       <c r="B109" s="3" t="inlineStr">
         <is>
-          <t>Spaced Practice: What Actually Makes It Stick</t>
+          <t>Spaced Practice: Retention Over Completion</t>
         </is>
       </c>
       <c r="C109" s="4" t="inlineStr">
@@ -5982,7 +5982,7 @@
       </c>
       <c r="B110" s="3" t="inlineStr">
         <is>
-          <t>Spaced Repetition System: Built to Prove Retention, Not Attendance</t>
+          <t>Spaced Repetition System: What to Look For</t>
         </is>
       </c>
       <c r="C110" s="4" t="inlineStr">
@@ -6131,7 +6131,7 @@
       </c>
       <c r="B113" s="3" t="inlineStr">
         <is>
-          <t>Spaced Repetition Benefits That Holds Up Under Pressure</t>
+          <t>The Real Payoff of Spaced Repetition for Teams</t>
         </is>
       </c>
       <c r="C113" s="4" t="inlineStr">
@@ -6178,7 +6178,7 @@
       </c>
       <c r="B114" s="3" t="inlineStr">
         <is>
-          <t>Frontline Leadership: Where Most Programs Break Down</t>
+          <t>Frontline Leadership Without the Training Fatigue</t>
         </is>
       </c>
       <c r="C114" s="4" t="inlineStr">
@@ -6229,7 +6229,7 @@
       </c>
       <c r="B115" s="3" t="inlineStr">
         <is>
-          <t>Frontline Managers: Retention Over Completion</t>
+          <t>Frontline Managers When the Pressure Is On</t>
         </is>
       </c>
       <c r="C115" s="4" t="inlineStr">
@@ -6276,7 +6276,7 @@
       </c>
       <c r="B116" s="3" t="inlineStr">
         <is>
-          <t>Training Management Solutions: Built for Readiness, Not Completion</t>
+          <t>Training Management Solutions: Built to Prove Retention, Not Attendance</t>
         </is>
       </c>
       <c r="C116" s="4" t="inlineStr">
@@ -6327,7 +6327,7 @@
       </c>
       <c r="B117" s="3" t="inlineStr">
         <is>
-          <t>Staff Online Training: What Actually Makes It Stick</t>
+          <t>Measuring the Impact of Staff Online Training</t>
         </is>
       </c>
       <c r="C117" s="4" t="inlineStr">
@@ -6374,7 +6374,7 @@
       </c>
       <c r="B118" s="3" t="inlineStr">
         <is>
-          <t>Choosing Corporate Training Tools for Zero-Fail Teams</t>
+          <t>Evaluating Corporate Training Tools for Mission-Critical Teams</t>
         </is>
       </c>
       <c r="C118" s="4" t="inlineStr">
@@ -6425,7 +6425,7 @@
       </c>
       <c r="B119" s="3" t="inlineStr">
         <is>
-          <t>Training Management Tool: What to Look For</t>
+          <t>Training Management Tool: Built for Readiness, Not Completion</t>
         </is>
       </c>
       <c r="C119" s="4" t="inlineStr">
@@ -6476,7 +6476,7 @@
       </c>
       <c r="B120" s="3" t="inlineStr">
         <is>
-          <t>Personalized Learning Pathways Without the Training Fatigue</t>
+          <t>Why Personalized Learning Pathways Won't Stick Without Reinforcement</t>
         </is>
       </c>
       <c r="C120" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Blank Slate: regenerate deck + workbook — Workforce pillar cleanup, LMS excluded
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/decks/blank-slate/keyword-research.xlsx
+++ b/decks/blank-slate/keyword-research.xlsx
@@ -697,23 +697,23 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Compliance Training Best Practices: Built to Prove Retention, Not Attendance</t>
+          <t>Compliance Training When the Pressure Is On</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>compliance training best practices</t>
+          <t>compliance training for managers</t>
         </is>
       </c>
       <c r="D3" s="5" t="n">
-        <v>90</v>
+        <v>110</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>13</v>
-      </c>
-      <c r="F3" s="6" t="inlineStr">
-        <is>
-          <t>Very Easy</t>
+        <v>23</v>
+      </c>
+      <c r="F3" s="8" t="inlineStr">
+        <is>
+          <t>Easy</t>
         </is>
       </c>
       <c r="G3" s="7" t="inlineStr">
@@ -723,12 +723,12 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Bottom of funnel</t>
+          <t>Middle of funnel</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Compare</t>
+          <t>Info</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -736,11 +736,7 @@
           <t>M1</t>
         </is>
       </c>
-      <c r="K3" s="3" t="inlineStr">
-        <is>
-          <t>Easy win — fast indexing expected. Commercial intent — direct buyer query</t>
-        </is>
-      </c>
+      <c r="K3" s="3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -748,23 +744,23 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Why Compliance Training Actually Matters</t>
+          <t>Compliance Training Best Practices: Built to Prove Retention, Not Attendance</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>why is compliance training important</t>
+          <t>compliance training best practices</t>
         </is>
       </c>
       <c r="D4" s="5" t="n">
         <v>90</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>24</v>
-      </c>
-      <c r="F4" s="8" t="inlineStr">
-        <is>
-          <t>Easy</t>
+        <v>13</v>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>Very Easy</t>
         </is>
       </c>
       <c r="G4" s="7" t="inlineStr">
@@ -774,12 +770,12 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Top of funnel</t>
+          <t>Bottom of funnel</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Info</t>
+          <t>Compare</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
@@ -787,7 +783,11 @@
           <t>M1</t>
         </is>
       </c>
-      <c r="K4" s="3" t="inlineStr"/>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t>Easy win — fast indexing expected. Commercial intent — direct buyer query</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -795,7 +795,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>New Employee Compliance Training When the Pressure Is On</t>
+          <t>Closing the Knowledge Gap in New Employee Compliance Training</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
@@ -897,7 +897,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Compliance Training for New Employees: Where Most Programs Break Down</t>
+          <t>Measuring the Impact of Compliance Training for New Employees</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -948,7 +948,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Training Compliance Tracking: Retention Over Completion</t>
+          <t>Making Training Compliance Tracking Stick for Frontline Teams</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -1050,7 +1050,7 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>The Science Behind Interactive Training</t>
+          <t>Why Interactive Training Won't Stick Without Reinforcement</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
@@ -1097,7 +1097,7 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Why Motivational Training Won't Stick Without Reinforcement</t>
+          <t>Turning Motivational Training Into Readiness You Can Prove</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
@@ -1148,7 +1148,7 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Rethinking Motivating Staff Training for Safety-Critical Teams</t>
+          <t>Motivating Staff Training Without the Training Fatigue</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
@@ -1250,7 +1250,7 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Corporate Gamification: Where Most Programs Break Down</t>
+          <t>Measuring the Impact of Corporate Gamification</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
@@ -1301,7 +1301,7 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Measuring the Impact of Gamification Features</t>
+          <t>Gamification Features: Retention Over Completion</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
@@ -1450,7 +1450,7 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Why Microlearning in Corporate Training Won't Stick Without Reinforcement</t>
+          <t>Turning Microlearning in Corporate Training Into Readiness You Can Prove</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
@@ -1501,7 +1501,7 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>Turning Creating Microlearning Content Into Readiness You Can Prove</t>
+          <t>Creating Microlearning Content: A Readiness-First Approach</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
@@ -1654,7 +1654,7 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>Rethinking Microlearning Strategies for Regulated Industries</t>
+          <t>Microlearning Strategies Without the Training Fatigue</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
@@ -1705,7 +1705,7 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>Gamified Microlearning Without the Training Fatigue</t>
+          <t>From Checkbox to Capability in Gamified Microlearning</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
@@ -1756,7 +1756,7 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>From Checkbox to Capability in Microlearning Gamification</t>
+          <t>Microlearning Gamification When the Pressure Is On</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
@@ -1807,7 +1807,7 @@
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>Microlearning Content Development When the Pressure Is On</t>
+          <t>Closing the Knowledge Gap in Microlearning Content Development</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
@@ -1905,7 +1905,7 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>Employee Retention Training: What Actually Makes It Stick</t>
+          <t>The Science Behind Employee Retention Training</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
@@ -1956,7 +1956,7 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>The Science Behind Training and Retention</t>
+          <t>Why Training and Retention Won't Stick Without Reinforcement</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
@@ -2105,7 +2105,7 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>Why Adult Learning Retention Won't Stick Without Reinforcement</t>
+          <t>Turning Adult Learning Retention Into Readiness You Can Prove</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
@@ -2156,7 +2156,7 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>Knowledge Retention After Training: A Readiness-First Approach</t>
+          <t>Rethinking Knowledge Retention After Training for Zero-Fail Teams</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
@@ -2207,7 +2207,7 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>Rethinking Knowledge Retention in the Workplace for Zero-Fail Teams</t>
+          <t>Knowledge Retention in the Workplace Without the Training Fatigue</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
@@ -2258,7 +2258,7 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>From Checkbox to Capability in Training Content Development</t>
+          <t>Closing the Knowledge Gap in Training Content Development</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
@@ -2309,19 +2309,19 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>Customized Training That Targets Real Knowledge Gaps</t>
+          <t>Tracking Employee Training: Retention Over Completion</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>customised training</t>
+          <t>tracking employee training</t>
         </is>
       </c>
       <c r="D35" s="5" t="n">
-        <v>90</v>
+        <v>140</v>
       </c>
       <c r="E35" s="2" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="F35" s="6" t="inlineStr">
         <is>
@@ -2360,19 +2360,19 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>Frontline Leadership Program: Retention Over Completion</t>
+          <t>Customized Training That Targets Real Knowledge Gaps</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>frontline leadership program</t>
+          <t>customised training</t>
         </is>
       </c>
       <c r="D36" s="5" t="n">
         <v>90</v>
       </c>
       <c r="E36" s="2" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F36" s="6" t="inlineStr">
         <is>
@@ -2411,19 +2411,19 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>Making Frontline Leadership Course Stick for High-Stakes Teams</t>
+          <t>How to Track Training</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>frontline leadership course</t>
+          <t>how to track training for employees</t>
         </is>
       </c>
       <c r="D37" s="5" t="n">
         <v>70</v>
       </c>
       <c r="E37" s="2" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="F37" s="6" t="inlineStr">
         <is>
@@ -2462,19 +2462,19 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>Turning Training for Frontline Staff Into Readiness You Can Prove</t>
+          <t>External Training Management System: Built to Prove Retention, Not Attendance</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>training for frontline staff</t>
+          <t>external training management system</t>
         </is>
       </c>
       <c r="D38" s="5" t="n">
-        <v>70</v>
+        <v>50</v>
       </c>
       <c r="E38" s="2" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F38" s="6" t="inlineStr">
         <is>
@@ -2488,12 +2488,12 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>Middle of funnel</t>
+          <t>Bottom of funnel</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>Info</t>
+          <t>Compare</t>
         </is>
       </c>
       <c r="J38" s="2" t="inlineStr">
@@ -2503,7 +2503,7 @@
       </c>
       <c r="K38" s="3" t="inlineStr">
         <is>
-          <t>Easy win — fast indexing expected</t>
+          <t>Easy win — fast indexing expected. Commercial intent — direct buyer query</t>
         </is>
       </c>
     </row>
@@ -2513,19 +2513,19 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>Choosing External Training Management System for Regulated Industries</t>
+          <t>How to Track Employee Training Progress</t>
         </is>
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>external training management system</t>
+          <t>how to track employee training progress</t>
         </is>
       </c>
       <c r="D39" s="5" t="n">
         <v>50</v>
       </c>
       <c r="E39" s="2" t="n">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="F39" s="6" t="inlineStr">
         <is>
@@ -2539,12 +2539,12 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>Bottom of funnel</t>
+          <t>Middle of funnel</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>Compare</t>
+          <t>Info</t>
         </is>
       </c>
       <c r="J39" s="2" t="inlineStr">
@@ -2554,7 +2554,7 @@
       </c>
       <c r="K39" s="3" t="inlineStr">
         <is>
-          <t>Easy win — fast indexing expected. Commercial intent — direct buyer query</t>
+          <t>Easy win — fast indexing expected</t>
         </is>
       </c>
     </row>
@@ -2564,7 +2564,7 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>Rethinking Frontline Worker Training for Compliance Teams</t>
+          <t>Turning Frontline Worker Training Into Readiness You Can Prove</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr">
@@ -2615,19 +2615,19 @@
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>Frontline Leadership Basic Principles Without the Training Fatigue</t>
+          <t>Keeping Staff Training on Track — and Retained</t>
         </is>
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>frontline leadership basic principles</t>
+          <t>track staff training</t>
         </is>
       </c>
       <c r="D41" s="5" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="E41" s="2" t="n">
-        <v>3</v>
+        <v>19</v>
       </c>
       <c r="F41" s="6" t="inlineStr">
         <is>
@@ -2905,19 +2905,19 @@
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>Running Compliance Training Through Your LMS: What Breaks</t>
+          <t>Why Compliance Training Actually Matters</t>
         </is>
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>learning management system for compliance training</t>
+          <t>why is compliance training important</t>
         </is>
       </c>
       <c r="D47" s="5" t="n">
         <v>90</v>
       </c>
       <c r="E47" s="2" t="n">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="F47" s="8" t="inlineStr">
         <is>
@@ -2931,7 +2931,7 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>Bottom of funnel</t>
+          <t>Top of funnel</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -2944,11 +2944,7 @@
           <t>M2</t>
         </is>
       </c>
-      <c r="K47" s="3" t="inlineStr">
-        <is>
-          <t>Commercial intent — direct buyer query</t>
-        </is>
-      </c>
+      <c r="K47" s="3" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
@@ -2956,7 +2952,7 @@
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>Closing the Knowledge Gap in Regulatory Compliance Training Courses</t>
+          <t>Regulatory Compliance Training Courses: Where Most Programs Break Down</t>
         </is>
       </c>
       <c r="C48" s="4" t="inlineStr">
@@ -3003,7 +2999,7 @@
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>Measuring the Impact of Regulatory Compliance Training Programs</t>
+          <t>Regulatory Compliance Training Programs: Retention Over Completion</t>
         </is>
       </c>
       <c r="C49" s="4" t="inlineStr">
@@ -3152,7 +3148,7 @@
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>Gamification for Employee Engagement: A Readiness-First Approach</t>
+          <t>Rethinking Gamification for Employee Engagement for Safety-Critical Teams</t>
         </is>
       </c>
       <c r="C52" s="4" t="inlineStr">
@@ -3250,7 +3246,7 @@
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>Employee Gamification Without the Training Fatigue</t>
+          <t>From Checkbox to Capability in Employee Gamification</t>
         </is>
       </c>
       <c r="C54" s="4" t="inlineStr">
@@ -3297,7 +3293,7 @@
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>From Checkbox to Capability in Employee Engagement Training</t>
+          <t>Employee Engagement Training When the Pressure Is On</t>
         </is>
       </c>
       <c r="C55" s="4" t="inlineStr">
@@ -3344,7 +3340,7 @@
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>Employee Engagement Training and Development: Retention Over Completion</t>
+          <t>Making Employee Engagement Training and Development Stick for Zero-Fail Teams</t>
         </is>
       </c>
       <c r="C56" s="4" t="inlineStr">
@@ -3391,7 +3387,7 @@
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>Making Gamified Features Stick for Zero-Fail Teams</t>
+          <t>Gamified Features, Reframed for Mission-Critical Teams</t>
         </is>
       </c>
       <c r="C57" s="4" t="inlineStr">
@@ -3438,7 +3434,7 @@
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>Choosing Microlearning Platform for Mission-Critical Teams</t>
+          <t>Choosing Microlearning Platform for High-Stakes Teams</t>
         </is>
       </c>
       <c r="C58" s="4" t="inlineStr">
@@ -3489,7 +3485,7 @@
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>Benefits of Microlearning, Reframed for High-Stakes Teams</t>
+          <t>The Science Behind Benefits of Microlearning</t>
         </is>
       </c>
       <c r="C59" s="4" t="inlineStr">
@@ -3638,7 +3634,7 @@
       </c>
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t>Corporate Microlearning: What Actually Makes It Stick</t>
+          <t>Why Corporate Microlearning Won't Stick Without Reinforcement</t>
         </is>
       </c>
       <c r="C62" s="4" t="inlineStr">
@@ -3736,7 +3732,7 @@
       </c>
       <c r="B64" s="3" t="inlineStr">
         <is>
-          <t>Microlearning Modules: A Readiness-First Approach</t>
+          <t>Rethinking Microlearning Modules for Regulated Industries</t>
         </is>
       </c>
       <c r="C64" s="4" t="inlineStr">
@@ -3783,7 +3779,7 @@
       </c>
       <c r="B65" s="3" t="inlineStr">
         <is>
-          <t>Closing the Knowledge Gap in Microlearning Resources</t>
+          <t>Microlearning Resources: Where Most Programs Break Down</t>
         </is>
       </c>
       <c r="C65" s="4" t="inlineStr">
@@ -3830,7 +3826,7 @@
       </c>
       <c r="B66" s="3" t="inlineStr">
         <is>
-          <t>Choosing Spaced Repetition App for Compliance Teams</t>
+          <t>Choosing Spaced Repetition App for Safety-Critical Teams</t>
         </is>
       </c>
       <c r="C66" s="4" t="inlineStr">
@@ -3881,7 +3877,7 @@
       </c>
       <c r="B67" s="3" t="inlineStr">
         <is>
-          <t>Making Learning Retention Stick for Safety-Critical Teams</t>
+          <t>Learning Retention, Reframed for Deskless Workforces</t>
         </is>
       </c>
       <c r="C67" s="4" t="inlineStr">
@@ -3928,7 +3924,7 @@
       </c>
       <c r="B68" s="3" t="inlineStr">
         <is>
-          <t>Knowledge Retention, Reframed for Deskless Workforces</t>
+          <t>Knowledge Retention: What Actually Makes It Stick</t>
         </is>
       </c>
       <c r="C68" s="4" t="inlineStr">
@@ -4073,7 +4069,7 @@
       </c>
       <c r="B71" s="3" t="inlineStr">
         <is>
-          <t>Turning Knowledge Retention Strategies Into Readiness You Can Prove</t>
+          <t>Knowledge Retention Strategies: A Readiness-First Approach</t>
         </is>
       </c>
       <c r="C71" s="4" t="inlineStr">
@@ -4214,23 +4210,23 @@
       </c>
       <c r="B74" s="3" t="inlineStr">
         <is>
-          <t>Closing the Knowledge Gap in Tracking Employee Training</t>
+          <t>Online Training When the Pressure Is On</t>
         </is>
       </c>
       <c r="C74" s="4" t="inlineStr">
         <is>
-          <t>tracking employee training</t>
+          <t>online training for employees</t>
         </is>
       </c>
       <c r="D74" s="5" t="n">
-        <v>140</v>
+        <v>320</v>
       </c>
       <c r="E74" s="2" t="n">
-        <v>18</v>
-      </c>
-      <c r="F74" s="6" t="inlineStr">
-        <is>
-          <t>Very Easy</t>
+        <v>34</v>
+      </c>
+      <c r="F74" s="8" t="inlineStr">
+        <is>
+          <t>Easy</t>
         </is>
       </c>
       <c r="G74" s="12" t="inlineStr">
@@ -4253,11 +4249,7 @@
           <t>M2</t>
         </is>
       </c>
-      <c r="K74" s="3" t="inlineStr">
-        <is>
-          <t>Easy win — fast indexing expected</t>
-        </is>
-      </c>
+      <c r="K74" s="3" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" s="2" t="n">
@@ -4265,23 +4257,23 @@
       </c>
       <c r="B75" s="3" t="inlineStr">
         <is>
-          <t>Frontline Leadership Skills: Where Most Programs Break Down</t>
+          <t>Making Personalized Learning Paths Stick for High-Stakes Teams</t>
         </is>
       </c>
       <c r="C75" s="4" t="inlineStr">
         <is>
-          <t>frontline leadership skills</t>
+          <t>personalized learning paths</t>
         </is>
       </c>
       <c r="D75" s="5" t="n">
         <v>140</v>
       </c>
       <c r="E75" s="2" t="n">
-        <v>18</v>
-      </c>
-      <c r="F75" s="6" t="inlineStr">
-        <is>
-          <t>Very Easy</t>
+        <v>32</v>
+      </c>
+      <c r="F75" s="8" t="inlineStr">
+        <is>
+          <t>Easy</t>
         </is>
       </c>
       <c r="G75" s="12" t="inlineStr">
@@ -4304,11 +4296,7 @@
           <t>M2</t>
         </is>
       </c>
-      <c r="K75" s="3" t="inlineStr">
-        <is>
-          <t>Easy win — fast indexing expected</t>
-        </is>
-      </c>
+      <c r="K75" s="3" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
@@ -4316,23 +4304,23 @@
       </c>
       <c r="B76" s="3" t="inlineStr">
         <is>
-          <t>Frontline Management Course, Reframed for Frontline Teams</t>
+          <t>Training Management Solutions: Built for Readiness, Not Completion</t>
         </is>
       </c>
       <c r="C76" s="4" t="inlineStr">
         <is>
-          <t>frontline management course</t>
+          <t>training management solutions</t>
         </is>
       </c>
       <c r="D76" s="5" t="n">
-        <v>70</v>
+        <v>110</v>
       </c>
       <c r="E76" s="2" t="n">
-        <v>14</v>
-      </c>
-      <c r="F76" s="6" t="inlineStr">
-        <is>
-          <t>Very Easy</t>
+        <v>28</v>
+      </c>
+      <c r="F76" s="8" t="inlineStr">
+        <is>
+          <t>Easy</t>
         </is>
       </c>
       <c r="G76" s="12" t="inlineStr">
@@ -4342,7 +4330,7 @@
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>Middle of funnel</t>
+          <t>Bottom of funnel</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
@@ -4357,7 +4345,7 @@
       </c>
       <c r="K76" s="3" t="inlineStr">
         <is>
-          <t>Easy win — fast indexing expected</t>
+          <t>Commercial intent — direct buyer query</t>
         </is>
       </c>
     </row>
@@ -4367,23 +4355,23 @@
       </c>
       <c r="B77" s="3" t="inlineStr">
         <is>
-          <t>Frontline Manager Training: What Actually Makes It Stick</t>
+          <t>Staff Online Training, Reframed for Frontline Teams</t>
         </is>
       </c>
       <c r="C77" s="4" t="inlineStr">
         <is>
-          <t>frontline manager training</t>
+          <t>staff online training</t>
         </is>
       </c>
       <c r="D77" s="5" t="n">
-        <v>70</v>
+        <v>110</v>
       </c>
       <c r="E77" s="2" t="n">
-        <v>14</v>
-      </c>
-      <c r="F77" s="6" t="inlineStr">
-        <is>
-          <t>Very Easy</t>
+        <v>21</v>
+      </c>
+      <c r="F77" s="8" t="inlineStr">
+        <is>
+          <t>Easy</t>
         </is>
       </c>
       <c r="G77" s="12" t="inlineStr">
@@ -4406,11 +4394,7 @@
           <t>M2</t>
         </is>
       </c>
-      <c r="K77" s="3" t="inlineStr">
-        <is>
-          <t>Easy win — fast indexing expected</t>
-        </is>
-      </c>
+      <c r="K77" s="3" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="2" t="n">
@@ -4418,23 +4402,23 @@
       </c>
       <c r="B78" s="3" t="inlineStr">
         <is>
-          <t>Frontline Employee Training: A Readiness-First Approach</t>
+          <t>Choosing Corporate Training Tools for Regulated Industries</t>
         </is>
       </c>
       <c r="C78" s="4" t="inlineStr">
         <is>
-          <t>frontline employee training</t>
+          <t>corporate training tools</t>
         </is>
       </c>
       <c r="D78" s="5" t="n">
-        <v>70</v>
+        <v>90</v>
       </c>
       <c r="E78" s="2" t="n">
-        <v>16</v>
-      </c>
-      <c r="F78" s="6" t="inlineStr">
-        <is>
-          <t>Very Easy</t>
+        <v>25</v>
+      </c>
+      <c r="F78" s="8" t="inlineStr">
+        <is>
+          <t>Easy</t>
         </is>
       </c>
       <c r="G78" s="12" t="inlineStr">
@@ -4444,7 +4428,7 @@
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>Middle of funnel</t>
+          <t>Bottom of funnel</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
@@ -4459,7 +4443,7 @@
       </c>
       <c r="K78" s="3" t="inlineStr">
         <is>
-          <t>Easy win — fast indexing expected</t>
+          <t>Commercial intent — direct buyer query</t>
         </is>
       </c>
     </row>
@@ -4469,23 +4453,23 @@
       </c>
       <c r="B79" s="3" t="inlineStr">
         <is>
-          <t>How to Track Employee Training Progress</t>
+          <t>Training Management Tool: What to Look For</t>
         </is>
       </c>
       <c r="C79" s="4" t="inlineStr">
         <is>
-          <t>how to track employee training progress</t>
+          <t>training management tool</t>
         </is>
       </c>
       <c r="D79" s="5" t="n">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="E79" s="2" t="n">
-        <v>18</v>
-      </c>
-      <c r="F79" s="6" t="inlineStr">
-        <is>
-          <t>Very Easy</t>
+        <v>26</v>
+      </c>
+      <c r="F79" s="8" t="inlineStr">
+        <is>
+          <t>Easy</t>
         </is>
       </c>
       <c r="G79" s="12" t="inlineStr">
@@ -4495,12 +4479,12 @@
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>Middle of funnel</t>
+          <t>Bottom of funnel</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>Info</t>
+          <t>Compare</t>
         </is>
       </c>
       <c r="J79" s="2" t="inlineStr">
@@ -4510,7 +4494,7 @@
       </c>
       <c r="K79" s="3" t="inlineStr">
         <is>
-          <t>Easy win — fast indexing expected</t>
+          <t>Commercial intent — direct buyer query</t>
         </is>
       </c>
     </row>
@@ -4520,23 +4504,23 @@
       </c>
       <c r="B80" s="3" t="inlineStr">
         <is>
-          <t>How to Keep Track of Employee Training</t>
+          <t>Evaluating Employee Training Video Platforms for Compliance Teams</t>
         </is>
       </c>
       <c r="C80" s="4" t="inlineStr">
         <is>
-          <t>how to keep track of training for employees</t>
+          <t>employee training video platforms</t>
         </is>
       </c>
       <c r="D80" s="5" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="E80" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="F80" s="6" t="inlineStr">
-        <is>
-          <t>Very Easy</t>
+        <v>30</v>
+      </c>
+      <c r="F80" s="8" t="inlineStr">
+        <is>
+          <t>Easy</t>
         </is>
       </c>
       <c r="G80" s="12" t="inlineStr">
@@ -4546,7 +4530,7 @@
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>Middle of funnel</t>
+          <t>Bottom of funnel</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
@@ -4561,7 +4545,7 @@
       </c>
       <c r="K80" s="3" t="inlineStr">
         <is>
-          <t>Easy win — fast indexing expected</t>
+          <t>Commercial intent — direct buyer query</t>
         </is>
       </c>
     </row>
@@ -4571,23 +4555,23 @@
       </c>
       <c r="B81" s="3" t="inlineStr">
         <is>
-          <t>Leadership Development for Frontline Supervisors: What to Look For</t>
+          <t>Rethinking Personalized Training Plans for Safety-Critical Teams</t>
         </is>
       </c>
       <c r="C81" s="4" t="inlineStr">
         <is>
-          <t>best leadership development training for frontline supervisors</t>
+          <t>personalized training plans</t>
         </is>
       </c>
       <c r="D81" s="5" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="E81" s="2" t="n">
-        <v>17</v>
-      </c>
-      <c r="F81" s="6" t="inlineStr">
-        <is>
-          <t>Very Easy</t>
+        <v>25</v>
+      </c>
+      <c r="F81" s="8" t="inlineStr">
+        <is>
+          <t>Easy</t>
         </is>
       </c>
       <c r="G81" s="12" t="inlineStr">
@@ -4597,12 +4581,12 @@
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>Bottom of funnel</t>
+          <t>Middle of funnel</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>Compare</t>
+          <t>Info</t>
         </is>
       </c>
       <c r="J81" s="2" t="inlineStr">
@@ -4610,11 +4594,7 @@
           <t>M2</t>
         </is>
       </c>
-      <c r="K81" s="3" t="inlineStr">
-        <is>
-          <t>Easy win — fast indexing expected. Commercial intent — direct buyer query</t>
-        </is>
-      </c>
+      <c r="K81" s="3" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" s="2" t="n">
@@ -5006,7 +4986,7 @@
       </c>
       <c r="B90" s="3" t="inlineStr">
         <is>
-          <t>Making Training and Employee Engagement Stick for Frontline Teams</t>
+          <t>Training and Employee Engagement, Reframed for Regulated Industries</t>
         </is>
       </c>
       <c r="C90" s="4" t="inlineStr">
@@ -5057,7 +5037,7 @@
       </c>
       <c r="B91" s="3" t="inlineStr">
         <is>
-          <t>Employee Engagement Courses, Reframed for Regulated Industries</t>
+          <t>Employee Engagement Courses: What Actually Makes It Stick</t>
         </is>
       </c>
       <c r="C91" s="4" t="inlineStr">
@@ -5104,7 +5084,7 @@
       </c>
       <c r="B92" s="3" t="inlineStr">
         <is>
-          <t>Gamification in the Workplace: What Actually Makes It Stick</t>
+          <t>The Science Behind Gamification in the Workplace</t>
         </is>
       </c>
       <c r="C92" s="4" t="inlineStr">
@@ -5202,7 +5182,7 @@
       </c>
       <c r="B94" s="3" t="inlineStr">
         <is>
-          <t>Turning Gamified Training Into Readiness You Can Prove</t>
+          <t>Gamified Training: A Readiness-First Approach</t>
         </is>
       </c>
       <c r="C94" s="4" t="inlineStr">
@@ -5300,7 +5280,7 @@
       </c>
       <c r="B96" s="3" t="inlineStr">
         <is>
-          <t>Interactive Training Modules When the Pressure Is On</t>
+          <t>Closing the Knowledge Gap in Interactive Training Modules</t>
         </is>
       </c>
       <c r="C96" s="4" t="inlineStr">
@@ -5347,7 +5327,7 @@
       </c>
       <c r="B97" s="3" t="inlineStr">
         <is>
-          <t>Closing the Knowledge Gap in Benefits of Gamification in the Workplace</t>
+          <t>Benefits of Gamification in the Workplace: Where Most Programs Break Down</t>
         </is>
       </c>
       <c r="C97" s="4" t="inlineStr">
@@ -5394,23 +5374,23 @@
       </c>
       <c r="B98" s="3" t="inlineStr">
         <is>
-          <t>Microlearning Apps: Built for Readiness, Not Completion</t>
+          <t>Microlearning: What Actually Makes It Stick</t>
         </is>
       </c>
       <c r="C98" s="4" t="inlineStr">
         <is>
-          <t>micro learning apps</t>
+          <t>micro learning</t>
         </is>
       </c>
       <c r="D98" s="5" t="n">
-        <v>1900</v>
+        <v>4400</v>
       </c>
       <c r="E98" s="2" t="n">
-        <v>27</v>
-      </c>
-      <c r="F98" s="8" t="inlineStr">
-        <is>
-          <t>Easy</t>
+        <v>52</v>
+      </c>
+      <c r="F98" s="13" t="inlineStr">
+        <is>
+          <t>Hard</t>
         </is>
       </c>
       <c r="G98" s="10" t="inlineStr">
@@ -5420,7 +5400,7 @@
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>Bottom of funnel</t>
+          <t>Middle of funnel</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
@@ -5435,7 +5415,7 @@
       </c>
       <c r="K98" s="3" t="inlineStr">
         <is>
-          <t>Pillar anchor — highest volume in Microlearning &amp; Delivery. Commercial intent — direct buyer query</t>
+          <t>Pillar anchor — highest volume in Microlearning &amp; Delivery</t>
         </is>
       </c>
     </row>
@@ -5445,23 +5425,23 @@
       </c>
       <c r="B99" s="3" t="inlineStr">
         <is>
-          <t>Microlearning: What It Is and Why It Matters</t>
+          <t>Microlearning Apps: Built for Readiness, Not Completion</t>
         </is>
       </c>
       <c r="C99" s="4" t="inlineStr">
         <is>
-          <t>what is microlearning</t>
+          <t>micro learning apps</t>
         </is>
       </c>
       <c r="D99" s="5" t="n">
-        <v>1000</v>
+        <v>1900</v>
       </c>
       <c r="E99" s="2" t="n">
-        <v>50</v>
-      </c>
-      <c r="F99" s="14" t="inlineStr">
-        <is>
-          <t>Moderate</t>
+        <v>27</v>
+      </c>
+      <c r="F99" s="8" t="inlineStr">
+        <is>
+          <t>Easy</t>
         </is>
       </c>
       <c r="G99" s="10" t="inlineStr">
@@ -5471,7 +5451,7 @@
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>Top of funnel</t>
+          <t>Bottom of funnel</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
@@ -5484,7 +5464,11 @@
           <t>M3</t>
         </is>
       </c>
-      <c r="K99" s="3" t="inlineStr"/>
+      <c r="K99" s="3" t="inlineStr">
+        <is>
+          <t>Commercial intent — direct buyer query</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="n">
@@ -5492,23 +5476,23 @@
       </c>
       <c r="B100" s="3" t="inlineStr">
         <is>
-          <t>Best Microlearning App: What to Look For</t>
+          <t>Microlearning: What It Is and Why It Matters</t>
         </is>
       </c>
       <c r="C100" s="4" t="inlineStr">
         <is>
-          <t>best micro learning app</t>
+          <t>what is microlearning</t>
         </is>
       </c>
       <c r="D100" s="5" t="n">
-        <v>390</v>
+        <v>1000</v>
       </c>
       <c r="E100" s="2" t="n">
-        <v>26</v>
-      </c>
-      <c r="F100" s="8" t="inlineStr">
-        <is>
-          <t>Easy</t>
+        <v>50</v>
+      </c>
+      <c r="F100" s="14" t="inlineStr">
+        <is>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="G100" s="10" t="inlineStr">
@@ -5518,12 +5502,12 @@
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>Bottom of funnel</t>
+          <t>Top of funnel</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t>Compare</t>
+          <t>Info</t>
         </is>
       </c>
       <c r="J100" s="2" t="inlineStr">
@@ -5531,11 +5515,7 @@
           <t>M3</t>
         </is>
       </c>
-      <c r="K100" s="3" t="inlineStr">
-        <is>
-          <t>Commercial intent — direct buyer query</t>
-        </is>
-      </c>
+      <c r="K100" s="3" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" s="2" t="n">
@@ -5543,16 +5523,16 @@
       </c>
       <c r="B101" s="3" t="inlineStr">
         <is>
-          <t>The Buyer's Guide to Microlearning Software</t>
+          <t>Best Microlearning App: What to Look For</t>
         </is>
       </c>
       <c r="C101" s="4" t="inlineStr">
         <is>
-          <t>microlearning software</t>
+          <t>best micro learning app</t>
         </is>
       </c>
       <c r="D101" s="5" t="n">
-        <v>260</v>
+        <v>390</v>
       </c>
       <c r="E101" s="2" t="n">
         <v>26</v>
@@ -5594,12 +5574,12 @@
       </c>
       <c r="B102" s="3" t="inlineStr">
         <is>
-          <t>Choosing a Microlearning Solution for Zero-Fail Teams</t>
+          <t>The Buyer's Guide to Microlearning Software</t>
         </is>
       </c>
       <c r="C102" s="4" t="inlineStr">
         <is>
-          <t>microlearning solution</t>
+          <t>microlearning software</t>
         </is>
       </c>
       <c r="D102" s="5" t="n">
@@ -5645,19 +5625,19 @@
       </c>
       <c r="B103" s="3" t="inlineStr">
         <is>
-          <t>Does Microlearning Actually Work?</t>
+          <t>Choosing a Microlearning Solution for Zero-Fail Teams</t>
         </is>
       </c>
       <c r="C103" s="4" t="inlineStr">
         <is>
-          <t>does microlearning work</t>
+          <t>microlearning solution</t>
         </is>
       </c>
       <c r="D103" s="5" t="n">
-        <v>210</v>
+        <v>260</v>
       </c>
       <c r="E103" s="2" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F103" s="8" t="inlineStr">
         <is>
@@ -5671,12 +5651,12 @@
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>Top of funnel</t>
+          <t>Bottom of funnel</t>
         </is>
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>Info</t>
+          <t>Compare</t>
         </is>
       </c>
       <c r="J103" s="2" t="inlineStr">
@@ -5684,7 +5664,11 @@
           <t>M3</t>
         </is>
       </c>
-      <c r="K103" s="3" t="inlineStr"/>
+      <c r="K103" s="3" t="inlineStr">
+        <is>
+          <t>Commercial intent — direct buyer query</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="n">
@@ -5692,19 +5676,19 @@
       </c>
       <c r="B104" s="3" t="inlineStr">
         <is>
-          <t>The Science Behind LMS Microlearning</t>
+          <t>Does Microlearning Actually Work?</t>
         </is>
       </c>
       <c r="C104" s="4" t="inlineStr">
         <is>
-          <t>lms microlearning</t>
+          <t>does microlearning work</t>
         </is>
       </c>
       <c r="D104" s="5" t="n">
-        <v>140</v>
+        <v>210</v>
       </c>
       <c r="E104" s="2" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F104" s="8" t="inlineStr">
         <is>
@@ -5718,7 +5702,7 @@
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>Middle of funnel</t>
+          <t>Top of funnel</t>
         </is>
       </c>
       <c r="I104" t="inlineStr">
@@ -5786,7 +5770,7 @@
       </c>
       <c r="B106" s="3" t="inlineStr">
         <is>
-          <t>Spaced Repetition: Where Most Programs Break Down</t>
+          <t>Measuring the Impact of Spaced Repetition</t>
         </is>
       </c>
       <c r="C106" s="4" t="inlineStr">
@@ -5837,7 +5821,7 @@
       </c>
       <c r="B107" s="3" t="inlineStr">
         <is>
-          <t>Measuring the Impact of Distributed Practice</t>
+          <t>Distributed Practice: Retention Over Completion</t>
         </is>
       </c>
       <c r="C107" s="4" t="inlineStr">
@@ -5935,7 +5919,7 @@
       </c>
       <c r="B109" s="3" t="inlineStr">
         <is>
-          <t>Spaced Practice: Retention Over Completion</t>
+          <t>Making Spaced Practice Stick for Compliance Teams</t>
         </is>
       </c>
       <c r="C109" s="4" t="inlineStr">
@@ -6178,23 +6162,23 @@
       </c>
       <c r="B114" s="3" t="inlineStr">
         <is>
-          <t>Frontline Leadership Without the Training Fatigue</t>
+          <t>From Checkbox to Capability in Employee Training</t>
         </is>
       </c>
       <c r="C114" s="4" t="inlineStr">
         <is>
-          <t>frontline leadership</t>
+          <t>employee training</t>
         </is>
       </c>
       <c r="D114" s="5" t="n">
-        <v>260</v>
+        <v>2900</v>
       </c>
       <c r="E114" s="2" t="n">
-        <v>19</v>
-      </c>
-      <c r="F114" s="6" t="inlineStr">
-        <is>
-          <t>Very Easy</t>
+        <v>75</v>
+      </c>
+      <c r="F114" s="13" t="inlineStr">
+        <is>
+          <t>Hard</t>
         </is>
       </c>
       <c r="G114" s="12" t="inlineStr">
@@ -6219,7 +6203,7 @@
       </c>
       <c r="K114" s="3" t="inlineStr">
         <is>
-          <t>Pillar anchor — highest volume in Workforce Training &amp; Readiness Measurement. Easy win — fast indexing expected</t>
+          <t>Pillar anchor — highest volume in Workforce Training &amp; Readiness Measurement</t>
         </is>
       </c>
     </row>
@@ -6229,23 +6213,23 @@
       </c>
       <c r="B115" s="3" t="inlineStr">
         <is>
-          <t>Frontline Managers When the Pressure Is On</t>
+          <t>Employee Training Management Software: Built to Prove Retention, Not Attendance</t>
         </is>
       </c>
       <c r="C115" s="4" t="inlineStr">
         <is>
-          <t>frontline managers</t>
+          <t>employee training management software</t>
         </is>
       </c>
       <c r="D115" s="5" t="n">
-        <v>170</v>
+        <v>590</v>
       </c>
       <c r="E115" s="2" t="n">
-        <v>22</v>
-      </c>
-      <c r="F115" s="8" t="inlineStr">
-        <is>
-          <t>Easy</t>
+        <v>51</v>
+      </c>
+      <c r="F115" s="13" t="inlineStr">
+        <is>
+          <t>Hard</t>
         </is>
       </c>
       <c r="G115" s="12" t="inlineStr">
@@ -6255,7 +6239,7 @@
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>Middle of funnel</t>
+          <t>Bottom of funnel</t>
         </is>
       </c>
       <c r="I115" t="inlineStr">
@@ -6268,7 +6252,11 @@
           <t>M3</t>
         </is>
       </c>
-      <c r="K115" s="3" t="inlineStr"/>
+      <c r="K115" s="3" t="inlineStr">
+        <is>
+          <t>Commercial intent — direct buyer query</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="n">
@@ -6276,23 +6264,23 @@
       </c>
       <c r="B116" s="3" t="inlineStr">
         <is>
-          <t>Training Management Solutions: Built to Prove Retention, Not Attendance</t>
+          <t>Evaluating Employee Development Platform for Mission-Critical Teams</t>
         </is>
       </c>
       <c r="C116" s="4" t="inlineStr">
         <is>
-          <t>training management solutions</t>
+          <t>employee development platform</t>
         </is>
       </c>
       <c r="D116" s="5" t="n">
-        <v>110</v>
+        <v>260</v>
       </c>
       <c r="E116" s="2" t="n">
-        <v>28</v>
-      </c>
-      <c r="F116" s="8" t="inlineStr">
-        <is>
-          <t>Easy</t>
+        <v>61</v>
+      </c>
+      <c r="F116" s="13" t="inlineStr">
+        <is>
+          <t>Hard</t>
         </is>
       </c>
       <c r="G116" s="12" t="inlineStr">
@@ -6327,23 +6315,23 @@
       </c>
       <c r="B117" s="3" t="inlineStr">
         <is>
-          <t>Measuring the Impact of Staff Online Training</t>
+          <t>Technical Skills Training: Where Most Programs Break Down</t>
         </is>
       </c>
       <c r="C117" s="4" t="inlineStr">
         <is>
-          <t>staff online training</t>
+          <t>technical skills training</t>
         </is>
       </c>
       <c r="D117" s="5" t="n">
-        <v>110</v>
+        <v>170</v>
       </c>
       <c r="E117" s="2" t="n">
-        <v>21</v>
-      </c>
-      <c r="F117" s="8" t="inlineStr">
-        <is>
-          <t>Easy</t>
+        <v>50</v>
+      </c>
+      <c r="F117" s="14" t="inlineStr">
+        <is>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="G117" s="12" t="inlineStr">
@@ -6374,23 +6362,23 @@
       </c>
       <c r="B118" s="3" t="inlineStr">
         <is>
-          <t>Evaluating Corporate Training Tools for Mission-Critical Teams</t>
+          <t>Measuring the Impact of Online Training Programs</t>
         </is>
       </c>
       <c r="C118" s="4" t="inlineStr">
         <is>
-          <t>corporate training tools</t>
+          <t>online training programs for employees</t>
         </is>
       </c>
       <c r="D118" s="5" t="n">
-        <v>90</v>
+        <v>170</v>
       </c>
       <c r="E118" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="F118" s="8" t="inlineStr">
-        <is>
-          <t>Easy</t>
+        <v>56</v>
+      </c>
+      <c r="F118" s="13" t="inlineStr">
+        <is>
+          <t>Hard</t>
         </is>
       </c>
       <c r="G118" s="12" t="inlineStr">
@@ -6400,7 +6388,7 @@
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>Bottom of funnel</t>
+          <t>Middle of funnel</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
@@ -6413,11 +6401,7 @@
           <t>M3</t>
         </is>
       </c>
-      <c r="K118" s="3" t="inlineStr">
-        <is>
-          <t>Commercial intent — direct buyer query</t>
-        </is>
-      </c>
+      <c r="K118" s="3" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" s="2" t="n">
@@ -6425,23 +6409,23 @@
       </c>
       <c r="B119" s="3" t="inlineStr">
         <is>
-          <t>Training Management Tool: Built for Readiness, Not Completion</t>
+          <t>Online Training Modules: What Actually Makes It Stick</t>
         </is>
       </c>
       <c r="C119" s="4" t="inlineStr">
         <is>
-          <t>training management tool</t>
+          <t>online training modules</t>
         </is>
       </c>
       <c r="D119" s="5" t="n">
-        <v>70</v>
+        <v>90</v>
       </c>
       <c r="E119" s="2" t="n">
-        <v>26</v>
-      </c>
-      <c r="F119" s="8" t="inlineStr">
-        <is>
-          <t>Easy</t>
+        <v>38</v>
+      </c>
+      <c r="F119" s="14" t="inlineStr">
+        <is>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="G119" s="12" t="inlineStr">
@@ -6451,12 +6435,12 @@
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>Bottom of funnel</t>
+          <t>Middle of funnel</t>
         </is>
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>Compare</t>
+          <t>Info</t>
         </is>
       </c>
       <c r="J119" s="2" t="inlineStr">
@@ -6464,11 +6448,7 @@
           <t>M3</t>
         </is>
       </c>
-      <c r="K119" s="3" t="inlineStr">
-        <is>
-          <t>Commercial intent — direct buyer query</t>
-        </is>
-      </c>
+      <c r="K119" s="3" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" s="2" t="n">
@@ -6476,23 +6456,23 @@
       </c>
       <c r="B120" s="3" t="inlineStr">
         <is>
-          <t>Why Personalized Learning Pathways Won't Stick Without Reinforcement</t>
+          <t>Why Corporate Training Management Won't Stick Without Reinforcement</t>
         </is>
       </c>
       <c r="C120" s="4" t="inlineStr">
         <is>
-          <t>personalized learning pathways</t>
+          <t>corporate training management</t>
         </is>
       </c>
       <c r="D120" s="5" t="n">
-        <v>70</v>
+        <v>90</v>
       </c>
       <c r="E120" s="2" t="n">
-        <v>29</v>
-      </c>
-      <c r="F120" s="8" t="inlineStr">
-        <is>
-          <t>Easy</t>
+        <v>50</v>
+      </c>
+      <c r="F120" s="14" t="inlineStr">
+        <is>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="G120" s="12" t="inlineStr">
@@ -6507,7 +6487,7 @@
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>Info</t>
+          <t>Compare</t>
         </is>
       </c>
       <c r="J120" s="2" t="inlineStr">
@@ -6523,23 +6503,23 @@
       </c>
       <c r="B121" s="3" t="inlineStr">
         <is>
-          <t>How to Track Training</t>
+          <t>Frontline Training: A Readiness-First Approach</t>
         </is>
       </c>
       <c r="C121" s="4" t="inlineStr">
         <is>
-          <t>how to track training for employees</t>
+          <t>front line training</t>
         </is>
       </c>
       <c r="D121" s="5" t="n">
-        <v>70</v>
+        <v>50</v>
       </c>
       <c r="E121" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="F121" s="6" t="inlineStr">
-        <is>
-          <t>Very Easy</t>
+        <v>37</v>
+      </c>
+      <c r="F121" s="14" t="inlineStr">
+        <is>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="G121" s="12" t="inlineStr">
@@ -6554,7 +6534,7 @@
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>Info</t>
+          <t>Compare</t>
         </is>
       </c>
       <c r="J121" s="2" t="inlineStr">
@@ -6562,11 +6542,7 @@
           <t>M3</t>
         </is>
       </c>
-      <c r="K121" s="3" t="inlineStr">
-        <is>
-          <t>Easy win — fast indexing expected</t>
-        </is>
-      </c>
+      <c r="K121" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -7084,9 +7060,9 @@
           <t>Info</t>
         </is>
       </c>
-      <c r="G15" s="15" t="inlineStr">
-        <is>
-          <t>Overflow</t>
+      <c r="G15" s="16" t="inlineStr">
+        <is>
+          <t>Yes (planned)</t>
         </is>
       </c>
     </row>
@@ -7150,9 +7126,9 @@
           <t>Compare</t>
         </is>
       </c>
-      <c r="G17" s="15" t="inlineStr">
-        <is>
-          <t>Overflow</t>
+      <c r="G17" s="16" t="inlineStr">
+        <is>
+          <t>Yes (planned)</t>
         </is>
       </c>
     </row>
@@ -9592,9 +9568,9 @@
           <t>Compare</t>
         </is>
       </c>
-      <c r="G91" s="15" t="inlineStr">
-        <is>
-          <t>Overflow</t>
+      <c r="G91" s="16" t="inlineStr">
+        <is>
+          <t>Yes (planned)</t>
         </is>
       </c>
     </row>
@@ -13057,9 +13033,9 @@
           <t>Info</t>
         </is>
       </c>
-      <c r="G196" s="15" t="inlineStr">
-        <is>
-          <t>Overflow</t>
+      <c r="G196" s="16" t="inlineStr">
+        <is>
+          <t>Yes (planned)</t>
         </is>
       </c>
     </row>
@@ -13849,9 +13825,9 @@
           <t>Info</t>
         </is>
       </c>
-      <c r="G220" s="16" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+      <c r="G220" s="15" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -14608,9 +14584,9 @@
           <t>Info</t>
         </is>
       </c>
-      <c r="G243" s="15" t="inlineStr">
-        <is>
-          <t>Overflow</t>
+      <c r="G243" s="16" t="inlineStr">
+        <is>
+          <t>Yes (planned)</t>
         </is>
       </c>
     </row>
@@ -18073,9 +18049,9 @@
           <t>Info</t>
         </is>
       </c>
-      <c r="G348" s="15" t="inlineStr">
-        <is>
-          <t>Overflow</t>
+      <c r="G348" s="16" t="inlineStr">
+        <is>
+          <t>Yes (planned)</t>
         </is>
       </c>
     </row>
@@ -18271,9 +18247,9 @@
           <t>Info</t>
         </is>
       </c>
-      <c r="G354" s="16" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+      <c r="G354" s="15" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -18403,9 +18379,9 @@
           <t>Info</t>
         </is>
       </c>
-      <c r="G358" s="15" t="inlineStr">
-        <is>
-          <t>Overflow</t>
+      <c r="G358" s="16" t="inlineStr">
+        <is>
+          <t>Yes (planned)</t>
         </is>
       </c>
     </row>
@@ -19987,9 +19963,9 @@
           <t>Info</t>
         </is>
       </c>
-      <c r="G406" s="16" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+      <c r="G406" s="15" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -20218,9 +20194,9 @@
           <t>Decision</t>
         </is>
       </c>
-      <c r="G413" s="15" t="inlineStr">
-        <is>
-          <t>Overflow</t>
+      <c r="G413" s="16" t="inlineStr">
+        <is>
+          <t>Yes (planned)</t>
         </is>
       </c>
     </row>
@@ -20482,9 +20458,9 @@
           <t>Info</t>
         </is>
       </c>
-      <c r="G421" s="16" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+      <c r="G421" s="15" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -21274,9 +21250,9 @@
           <t>Info</t>
         </is>
       </c>
-      <c r="G445" s="15" t="inlineStr">
-        <is>
-          <t>Overflow</t>
+      <c r="G445" s="16" t="inlineStr">
+        <is>
+          <t>Yes (planned)</t>
         </is>
       </c>
     </row>
@@ -23914,9 +23890,9 @@
           <t>Decision</t>
         </is>
       </c>
-      <c r="G525" s="16" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+      <c r="G525" s="15" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -23947,9 +23923,9 @@
           <t>Compare</t>
         </is>
       </c>
-      <c r="G526" s="15" t="inlineStr">
-        <is>
-          <t>Overflow</t>
+      <c r="G526" s="16" t="inlineStr">
+        <is>
+          <t>Yes (planned)</t>
         </is>
       </c>
     </row>
@@ -24673,9 +24649,9 @@
           <t>Info</t>
         </is>
       </c>
-      <c r="G548" s="16" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+      <c r="G548" s="15" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -26224,9 +26200,9 @@
           <t>Info</t>
         </is>
       </c>
-      <c r="G595" s="15" t="inlineStr">
-        <is>
-          <t>Overflow</t>
+      <c r="G595" s="16" t="inlineStr">
+        <is>
+          <t>Yes (planned)</t>
         </is>
       </c>
     </row>
@@ -29161,9 +29137,9 @@
           <t>Decision</t>
         </is>
       </c>
-      <c r="G684" s="16" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+      <c r="G684" s="15" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -29194,9 +29170,9 @@
           <t>Info</t>
         </is>
       </c>
-      <c r="G685" s="16" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+      <c r="G685" s="15" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -29227,9 +29203,9 @@
           <t>Info</t>
         </is>
       </c>
-      <c r="G686" s="16" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+      <c r="G686" s="15" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -31801,9 +31777,9 @@
           <t>Decision</t>
         </is>
       </c>
-      <c r="G764" s="16" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+      <c r="G764" s="15" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -32296,9 +32272,9 @@
           <t>Info</t>
         </is>
       </c>
-      <c r="G779" s="16" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+      <c r="G779" s="15" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -32329,9 +32305,9 @@
           <t>Info</t>
         </is>
       </c>
-      <c r="G780" s="16" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+      <c r="G780" s="15" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -34474,9 +34450,9 @@
           <t>Compare</t>
         </is>
       </c>
-      <c r="G845" s="15" t="inlineStr">
-        <is>
-          <t>Overflow</t>
+      <c r="G845" s="16" t="inlineStr">
+        <is>
+          <t>Yes (planned)</t>
         </is>
       </c>
     </row>
@@ -38540,7 +38516,7 @@
     <row r="14" ht="60" customHeight="1">
       <c r="A14" s="21" t="inlineStr">
         <is>
-          <t>The plan runs roughly 8% awareness / 67% consideration / 25% decision.
+          <t>The plan runs roughly 8% awareness / 66% consideration / 26% decision.
 Weighted toward the middle of the funnel — the 'how do I fix retention' searches where buyers compare approaches and Blank Slate's proof does the most work.
 The plan is deliberately on-brand: it never positions Blank Slate as an LMS, e-learning, or 'training software'.</t>
         </is>

</xml_diff>